<commit_message>
Label creator games by element name instead of side 1/2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJR2Tn3kCW9FarCETGMuGF
</commit_message>
<xml_diff>
--- a/data/audience_and_creators.xlsx
+++ b/data/audience_and_creators.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YouTube: по 50 самых просматриваемых видео (категория «Игры») на каждую игру. На стыке — канал, снимавший игру-гибрид или игры обеих сторон. Официальные каналы и трейлеры исключены.</t>
+          <t>YouTube: по 50 самых просматриваемых видео (категория «Игры») на каждую игру. На стыке — канал, снимавший игру-гибрид или игры обоих элементов стыка. В скобках у игры — её элемент: например, [охота], [френдслоп] или [гибрид] (оба сразу). Официальные каналы и трейлеры исключены.</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Игры (сторона стыка)</t>
+          <t>Игры [элемент]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Pratfall [гибрид]; Splitgate [сторона 2]</t>
+          <t>Lethal Company [френдслоп]; Pratfall [гибрид]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Saints Row: The Third [сторона 2]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Saints Row: The Third [френдслоп]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Pratfall [гибрид]</t>
+          <t>Lethal Company [френдслоп]; Pratfall [гибрид]</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Pratfall [гибрид]</t>
+          <t>Lethal Company [френдслоп]; Pratfall [гибрид]</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pratfall [гибрид]; Splitgate [сторона 2]</t>
+          <t>Pratfall [гибрид]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Necromunda: Hired Gun [сторона 1]; Splitgate [сторона 2]</t>
+          <t>Necromunda: Hired Gun [собака]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pratfall [гибрид]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Pratfall [гибрид]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Saints Row IV: Re-Elected [сторона 2]; Saints Row: The Third [сторона 2]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Saints Row IV: Re-Elected [френдслоп]; Saints Row: The Third [френдслоп]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Saints Row: The Third [сторона 2]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Saints Row: The Third [френдслоп]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Pratfall [гибрид]; Splitgate [сторона 2]</t>
+          <t>Pratfall [гибрид]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Saints Row: The Third [сторона 2]; Necromunda: Hired Gun [сторона 1]; Saints Row IV: Re-Elected [сторона 2]</t>
+          <t>Saints Row: The Third [френдслоп]; Necromunda: Hired Gun [собака]; Saints Row IV: Re-Elected [френдслоп]</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PHOGS! [гибрид]; Nickelodeon All-Star Brawl [сторона 1]</t>
+          <t>PHOGS! [гибрид]; Nickelodeon All-Star Brawl [собака]</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Pratfall [гибрид]; Splitgate [сторона 2]</t>
+          <t>Pratfall [гибрид]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Splitgate [сторона 2]; Montaro [сторона 1]; Super Auto Pets [сторона 1]</t>
+          <t>Splitgate [френдслоп]; Montaro [собака]; Super Auto Pets [собака]</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Saints Row: The Third [сторона 2]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Saints Row: The Third [френдслоп]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PHOGS! [гибрид]; Cat Quest II [сторона 1]</t>
+          <t>PHOGS! [гибрид]; Cat Quest II [собака]</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Nickelodeon All-Star Brawl [сторона 1]; Splitgate [сторона 2]</t>
+          <t>Nickelodeon All-Star Brawl [собака]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Pratfall [гибрид]</t>
+          <t>Lethal Company [френдслоп]; Pratfall [гибрид]</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -3947,7 +3947,7 @@
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Cat Quest II [сторона 1]; PHOGS! [гибрид]</t>
+          <t>Cat Quest II [собака]; PHOGS! [гибрид]</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Игры (сторона стыка)</t>
+          <t>Игры [элемент]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; 7 Days to Die [сторона 2]; Blair Witch [гибрид]; Killing Floor 2 [сторона 2]</t>
+          <t>Lethal Company [хоррор]; 7 Days to Die [хоррор]; Blair Witch [гибрид]; Killing Floor 2 [хоррор]</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Dying Light [сторона 2]; Blair Witch [гибрид]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Dying Light [хоррор]; Blair Witch [гибрид]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Blair Witch [гибрид]; Dying Light [сторона 2]</t>
+          <t>Blair Witch [гибрид]; Dying Light [хоррор]</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; PEAK [сторона 2]; Blair Witch [гибрид]</t>
+          <t>Lethal Company [хоррор]; PEAK [хоррор]; Blair Witch [гибрид]</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sakura Spirit [сторона 1]; Blair Witch [гибрид]</t>
+          <t>Sakura Spirit [собака]; Blair Witch [гибрид]</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Dying Light [сторона 2]; Blair Witch [гибрид]</t>
+          <t>Dying Light [хоррор]; Blair Witch [гибрид]</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -5582,7 +5582,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Dying Light [сторона 2]; Blair Witch [гибрид]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Dying Light [хоррор]; Blair Witch [гибрид]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Dying Light [сторона 2]; Blair Witch [гибрид]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Dying Light [хоррор]; Blair Witch [гибрид]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Blair Witch [гибрид]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Blair Witch [гибрид]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Blair Witch [гибрид]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Blair Witch [гибрид]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Necromunda: Hired Gun [сторона 1]; Killing Floor 2 [сторона 2]</t>
+          <t>Necromunda: Hired Gun [собака]; Killing Floor 2 [хоррор]</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Killing Floor 2 [сторона 2]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Killing Floor 2 [хоррор]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Игры (сторона стыка)</t>
+          <t>Игры [элемент]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sakura Spirit [сторона 1]; Blair Witch [сторона 1]; Dinosaur Hunt [сторона 2]</t>
+          <t>Sakura Spirit [собака]; Blair Witch [собака]; Dinosaur Hunt [охота]</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -9727,7 +9727,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Adore [гибрид]; WolfQuest: Anniversary Edition [сторона 2]</t>
+          <t>Adore [гибрид]; WolfQuest: Anniversary Edition [охота]</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -9799,7 +9799,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hunting Simulator 2 [гибрид]; Super Auto Pets [сторона 1]</t>
+          <t>Hunting Simulator 2 [гибрид]; Super Auto Pets [собака]</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Hunting Simulator 2 [гибрид]; WolfQuest: Anniversary Edition [сторона 2]</t>
+          <t>Hunting Simulator 2 [гибрид]; WolfQuest: Anniversary Edition [охота]</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -10331,7 +10331,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Adore [гибрид]; DYSMANTLE [сторона 2]; Necromunda: Hired Gun [сторона 1]</t>
+          <t>Adore [гибрид]; DYSMANTLE [охота]; Necromunda: Hired Gun [собака]</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Adore [гибрид]; DYSMANTLE [сторона 2]; Ice World [гибрид]</t>
+          <t>Adore [гибрид]; DYSMANTLE [охота]; Ice World [гибрид]</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>theHunter: Call of the Wild™ [сторона 2]; Way of the Hunter 2 [гибрид]; Hunting Simulator 2 [гибрид]</t>
+          <t>theHunter: Call of the Wild™ [охота]; Way of the Hunter 2 [гибрид]; Hunting Simulator 2 [гибрид]</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -10899,7 +10899,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>theHunter: Call of the Wild™ [сторона 2]; Hunting Simulator 2 [гибрид]; Way of the Hunter 2 [гибрид]</t>
+          <t>theHunter: Call of the Wild™ [охота]; Hunting Simulator 2 [гибрид]; Way of the Hunter 2 [гибрид]</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>theHunter: Call of the Wild™ [сторона 2]; Way of the Hunter 2 [гибрид]</t>
+          <t>theHunter: Call of the Wild™ [охота]; Way of the Hunter 2 [гибрид]</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -12574,7 +12574,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Игры (сторона стыка)</t>
+          <t>Игры [элемент]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Rake [гибрид]; Depth [сторона 1]; R.E.P.O. [сторона 2]; Killing Floor [сторона 2]</t>
+          <t>Lethal Company [френдслоп]; Rake [гибрид]; Depth [охота]; R.E.P.O. [френдслоп]; Killing Floor [френдслоп]</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -12682,7 +12682,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>R.E.P.O. [сторона 2]; Rake [гибрид]</t>
+          <t>R.E.P.O. [френдслоп]; Rake [гибрид]</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -12858,7 +12858,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Depth [сторона 1]; Lethal Company [сторона 2]</t>
+          <t>Depth [охота]; Lethal Company [френдслоп]</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -12894,7 +12894,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>R.E.P.O. [сторона 2]; Rake [гибрид]</t>
+          <t>R.E.P.O. [френдслоп]; Rake [гибрид]</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>R.E.P.O. [сторона 2]; Lethal Company [сторона 2]; Depth [сторона 1]</t>
+          <t>R.E.P.O. [френдслоп]; Lethal Company [френдслоп]; Depth [охота]</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -13142,7 +13142,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; R.E.P.O. [сторона 2]; Ranch Simulator: Build, Hunt, Farm [сторона 1]; PAYDAY 2 [сторона 2]</t>
+          <t>Lethal Company [френдслоп]; R.E.P.O. [френдслоп]; Ranch Simulator: Build, Hunt, Farm [охота]; PAYDAY 2 [френдслоп]</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -13250,7 +13250,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Rake [гибрид]; Depth [сторона 1]</t>
+          <t>Rake [гибрид]; Depth [охота]</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Rake [гибрид]; Splitgate [сторона 2]</t>
+          <t>Rake [гибрид]; Splitgate [френдслоп]</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Игры (сторона стыка)</t>
+          <t>Игры [элемент]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -13925,7 +13925,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Rake [гибрид]; 7 Days to Die [сторона 2]; Depth [гибрид]; Killing Floor 2 [сторона 2]</t>
+          <t>Lethal Company [хоррор]; Rake [гибрид]; 7 Days to Die [хоррор]; Depth [гибрид]; Killing Floor 2 [хоррор]</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -14029,7 +14029,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rake [гибрид]; Killing Floor 2 [сторона 2]</t>
+          <t>Rake [гибрид]; Killing Floor 2 [хоррор]</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Depth [гибрид]; Lethal Company [сторона 2]</t>
+          <t>Depth [гибрид]; Lethal Company [хоррор]</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -14273,7 +14273,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Depth [гибрид]; Dying Light [сторона 2]</t>
+          <t>Depth [гибрид]; Dying Light [хоррор]</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -14381,7 +14381,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Night of the Dead [гибрид]; DYSMANTLE [сторона 1]</t>
+          <t>Night of the Dead [гибрид]; DYSMANTLE [охота]</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Depth [гибрид]</t>
+          <t>Lethal Company [хоррор]; Depth [гибрид]</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -14801,7 +14801,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Lethal Company [сторона 2]; Ranch Simulator: Build, Hunt, Farm [сторона 1]</t>
+          <t>Lethal Company [хоррор]; Ranch Simulator: Build, Hunt, Farm [охота]</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -14981,7 +14981,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>7 Days to Die [сторона 2]; Ranch Simulator: Build, Hunt, Farm [сторона 1]; The Isle [гибрид]; Night of the Dead [гибрид]</t>
+          <t>7 Days to Die [хоррор]; Ranch Simulator: Build, Hunt, Farm [охота]; The Isle [гибрид]; Night of the Dead [гибрид]</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>7 Days to Die [сторона 2]; Killing Floor 2 [сторона 2]; Depth [гибрид]</t>
+          <t>7 Days to Die [хоррор]; Killing Floor 2 [хоррор]; Depth [гибрид]</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -15593,7 +15593,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DYSMANTLE [сторона 1]; Night of the Dead [гибрид]</t>
+          <t>DYSMANTLE [охота]; Night of the Dead [гибрид]</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -15913,7 +15913,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Night of the Dead [гибрид]; DYSMANTLE [сторона 1]</t>
+          <t>Night of the Dead [гибрид]; DYSMANTLE [охота]</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -16409,7 +16409,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>7 Days to Die [сторона 2]; Night of the Dead [гибрид]</t>
+          <t>7 Days to Die [хоррор]; Night of the Dead [гибрид]</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Сторона</t>
+          <t>Элемент</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18016,7 +18016,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -18042,7 +18042,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -18068,7 +18068,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -18094,7 +18094,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -18120,7 +18120,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -18146,7 +18146,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -18172,7 +18172,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -18224,7 +18224,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -18316,7 +18316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -18368,7 +18368,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -18394,7 +18394,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -18420,7 +18420,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -18446,7 +18446,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -18472,7 +18472,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -18498,7 +18498,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -18524,7 +18524,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -18550,7 +18550,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>френдслоп</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -18686,7 +18686,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -18712,7 +18712,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -18738,7 +18738,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -18764,7 +18764,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -18790,7 +18790,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -18816,7 +18816,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -18868,7 +18868,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -18894,7 +18894,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -18920,7 +18920,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -19056,7 +19056,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -19082,7 +19082,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -19108,7 +19108,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -19134,7 +19134,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -19160,7 +19160,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>охота</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -19186,7 +19186,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -19238,7 +19238,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -19264,7 +19264,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -19290,7 +19290,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -19426,7 +19426,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -19452,7 +19452,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -19478,7 +19478,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -19530,7 +19530,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>сторона 1</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -19556,7 +19556,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -19582,7 +19582,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -19608,7 +19608,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -19634,7 +19634,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -19660,7 +19660,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>сторона 2</t>
+          <t>хоррор</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">

</xml_diff>